<commit_message>
Finalize Verstapost evidence and test analysis
</commit_message>
<xml_diff>
--- a/docs/milestones/VERSTAPOST_REQUIREMENTS_TRACKER.xlsx
+++ b/docs/milestones/VERSTAPOST_REQUIREMENTS_TRACKER.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M46"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1187,22 +1187,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t/>
+          <t>+</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Fix / measure</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t/>
+          <t>ToF calibration note</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ToF accuracy is measured but shows large offset/error; calibration needed</t>
+          <t>Offset measured and documented; correction model valid for 50-300 mm short/medium obstacle logic; retest after final mounting.</t>
         </is>
       </c>
     </row>
@@ -1252,22 +1252,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t/>
+          <t>+</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Fix / measure</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t/>
+          <t>PCB evidence check</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1292,12 +1292,12 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t/>
+          <t>Latest Gerber/drill archive 2026-06-17</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>add DRC/export screenshot if available</t>
+          <t>Closed: schematic/layout PNG+JSON, 3D PCB screenshot, and latest 2026-06-17 Gerber/drill manufacturing archive are present. DRC screenshot remains optional production evidence.</t>
         </is>
       </c>
     </row>
@@ -1317,22 +1317,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t/>
+          <t>+</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Fix / measure</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1347,22 +1347,22 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t/>
+          <t>Power brownout analysis</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t/>
+          <t>Power brownout retest 2026-06-17</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t/>
+          <t>Power brownout retest summary</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>main controller stayed up in test; camera endpoint failures still need retest</t>
+          <t>Closed for documented operating range PWM 80-180: final retest has 30/30 rows with reset=no and Wi-Fi disconnect=no; browser camera observed during test. PWM 255 is documented as outside stable operating range.</t>
         </is>
       </c>
     </row>
@@ -1642,22 +1642,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t/>
+          <t>+</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Fix / measure</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1667,27 +1667,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t/>
+          <t>Tap-drive algorithm</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t/>
+          <t>Camera calibration and tap-drive plan</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t/>
+          <t>Tap-drive accuracy template</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t/>
+          <t>Tap-drive accuracy summary</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>calibrate camera; measure target accuracy</t>
+          <t>Closed: timed tap-drive algorithm measured in 5 physical trials; 5/5 pass, median error 20 mm, max error 141.4 mm. Red servo disabled; future improvement is pixel logging/homography calibration.</t>
         </is>
       </c>
     </row>
@@ -1707,52 +1707,52 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t/>
+          <t>+</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t/>
+          <t>Camera calibration and tap-drive plan</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t/>
+          <t>Camera calibration notebook</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t/>
+          <t>Executed camera calibration notebook</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t/>
+          <t>Homography calibration summary</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t/>
+          <t>Camera homography JSON/residuals</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>add OpenCV notebook/calibration file</t>
+          <t>Closed: UI CALIB mode used to collect 6 real Cam1 homography points; generated pixel-to-arena JSON with median residual 45.0 mm and max 68.3 mm. Chessboard intrinsics remain optional future precision improvement.</t>
         </is>
       </c>
     </row>
@@ -1772,52 +1772,52 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t/>
+          <t>+</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Fix / measure</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t/>
+          <t>Cam2 color firmware</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t/>
+          <t>Color repeatability CSV</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t/>
+          <t>Color repeatability summary</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t/>
+          <t>TCS34725 purchase evidence Order3</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t/>
+          <t>Firmware UI screenshots</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>implement closed-loop retreat/avoid behavior or document diagnostic-only status</t>
+          <t>Closed: Cam2 TCS34725 telemetry measured on red/light/dark surfaces; classifier threshold fixed and flashed; UI confirmed COLOR DARK; purchase and UI screenshot evidence added. Closed-loop color retreat is not claimed.</t>
         </is>
       </c>
     </row>
@@ -1857,32 +1857,32 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>main UI</t>
+          <t>Auto behavior code</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t/>
+          <t>Auto behavior logger</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t/>
+          <t>Auto behavior observation</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t/>
+          <t>Operator observation CSV</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t/>
+          <t>Auto logger UI screenshot</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>add measured reliability tests</t>
+          <t>Partial: auto logger implemented, UI screenshots and video evidence indexed; operator observed turn/avoid at about 200 mm; battery depleted before full 5-trial logger CSV. Need charged robot run to close reliability claim.</t>
         </is>
       </c>
     </row>
@@ -2382,27 +2382,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/README.md</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/Image (1).jpg</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/Mutimedia.jpg</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/PXL_20260613_160049625.jpg</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>add final photo set</t>
+          <t>Partial: fabrication, electronics integration, printed enclosure, and assembled robot photos are indexed. Still add final multi-angle front/back/left/right/top photos for a stronger final package.</t>
         </is>
       </c>
     </row>
@@ -2772,27 +2772,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/README.md</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/Image (1).jpg</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/Mutimedia.jpg</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/PXL_20260613_160049625.jpg</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>add final photos and measured service checks</t>
+          <t>Partial: assembly checklist and photo evidence are present. Still add final multi-angle photos plus battery service and endurance measurements.</t>
         </is>
       </c>
     </row>
@@ -2902,27 +2902,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/Image.jpg</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/Image (2).jpg</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/PXL_20260613_160049625.jpg</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/assets/photos/README.md</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>validate material-specific values on the final print</t>
+          <t>Partial: printed-part photo evidence is present. Still validate final material-specific heat, impact, battery-service, and endurance results.</t>
         </is>
       </c>
     </row>
@@ -3059,93 +3059,96 @@
   </sheetData>
   <autoFilter ref="A1:M46"/>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
-    <hyperlink ref="I2" r:id="rId2" tooltip="Versta1.png -&gt; ../assets/briefs/Versta1.png"/>
-    <hyperlink ref="H3" r:id="rId3" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
-    <hyperlink ref="I3" r:id="rId4" tooltip="system_block.drawio.png -&gt; ../../hardware/diagrams/system_block.drawio.png"/>
-    <hyperlink ref="H4" r:id="rId5" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
-    <hyperlink ref="I4" r:id="rId6" tooltip="TECH_COMPARISON.md -&gt; ../specification/TECH_COMPARISON.md"/>
-    <hyperlink ref="H5" r:id="rId7" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
-    <hyperlink ref="H6" r:id="rId8" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
-    <hyperlink ref="H7" r:id="rId9" tooltip="BOM.csv -&gt; ../specification/BOM.csv"/>
-    <hyperlink ref="I7" r:id="rId10" tooltip="Order1.png -&gt; ../assets/orders/Order1.png"/>
-    <hyperlink ref="J7" r:id="rId11" tooltip="Order2.png -&gt; ../assets/orders/Order2.png"/>
-    <hyperlink ref="H8" r:id="rId12" tooltip="power_scheme.md -&gt; ../specification/power_scheme.md"/>
-    <hyperlink ref="I8" r:id="rId13" tooltip="power_tree.drawio.png -&gt; ../../hardware/diagrams/power_tree.drawio.png"/>
-    <hyperlink ref="J8" r:id="rId14" tooltip="power_brownout_test.csv -&gt; ../../tests/results/power_brownout_test.csv"/>
-    <hyperlink ref="H9" r:id="rId15" tooltip="test_plan.md -&gt; ../testing/test_plan.md"/>
-    <hyperlink ref="H10" r:id="rId16" tooltip="hardware/cad/ver1 -&gt; ../../hardware/cad/ver1"/>
-    <hyperlink ref="I10" r:id="rId17" tooltip="hardware/pcb/README.md -&gt; ../../hardware/pcb/README.md"/>
-    <hyperlink ref="J10" r:id="rId18" tooltip="main -&gt; ../../firmware/main"/>
-    <hyperlink ref="K10" r:id="rId19" tooltip="cam -&gt; ../../firmware/camera/sketch_jan17a"/>
-    <hyperlink ref="H11" r:id="rId20" tooltip="TECH_COMPARISON.md -&gt; ../specification/TECH_COMPARISON.md"/>
-    <hyperlink ref="I11" r:id="rId21" tooltip="Vordlev_analyys_summary.md -&gt; ../analysis/Vordlev_analyys_summary.md"/>
-    <hyperlink ref="J11" r:id="rId22" tooltip="Vordlev_analyys.docx -&gt; ../analysis/Vordlev_analyys.docx"/>
-    <hyperlink ref="H12" r:id="rId23" tooltip="main firmware -&gt; ../../firmware/main/main.ino"/>
-    <hyperlink ref="I12" r:id="rId24" tooltip="web UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="J12" r:id="rId25" tooltip="motion logic -&gt; ../../firmware/main/02_Motion.ino"/>
-    <hyperlink ref="H13" r:id="rId26" tooltip="main firmware -&gt; ../../firmware/main/main.ino"/>
-    <hyperlink ref="I13" r:id="rId27" tooltip="web handlers -&gt; ../../firmware/main/03_WebHandlers.ino"/>
-    <hyperlink ref="H14" r:id="rId28" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="I14" r:id="rId29" tooltip="movement_speed_test.csv -&gt; ../../tests/results/movement_speed_test.csv"/>
-    <hyperlink ref="H15" r:id="rId30" tooltip="movement_speed_test.csv -&gt; ../../tests/results/movement_speed_test.csv"/>
-    <hyperlink ref="I15" r:id="rId31" tooltip="movement_drift_test.csv -&gt; ../../tests/results/movement_drift_test.csv"/>
-    <hyperlink ref="J15" r:id="rId32" tooltip="movement_turn_test.csv -&gt; ../../tests/results/movement_turn_test.csv"/>
-    <hyperlink ref="K15" r:id="rId33" tooltip="tof_stop_test.csv -&gt; ../../tests/results/tof_stop_test.csv"/>
-    <hyperlink ref="H16" r:id="rId34" tooltip="http_latency_analysis.ipynb -&gt; ../../tests/notebooks/http_latency_analysis.ipynb"/>
-    <hyperlink ref="I16" r:id="rId35" tooltip="latency_test_result.md -&gt; ../testing/latency_test_result.md"/>
-    <hyperlink ref="J16" r:id="rId36" tooltip="test_results_analysis.ipynb -&gt; ../../tests/notebooks/test_results_analysis.ipynb"/>
-    <hyperlink ref="H17" r:id="rId37" tooltip="camera firmware -&gt; ../../firmware/camera/sketch_jan17a/sketch_jan17a.ino"/>
-    <hyperlink ref="I17" r:id="rId38" tooltip="demo video -&gt; ../../media/video/MicrosoftTeams-video.mp4"/>
-    <hyperlink ref="H18" r:id="rId39" tooltip="main firmware -&gt; ../../firmware/main/main.ino"/>
-    <hyperlink ref="I18" r:id="rId40" tooltip="tof_stop_test.csv -&gt; ../../tests/results/tof_stop_test.csv"/>
-    <hyperlink ref="J18" r:id="rId41" tooltip="tof_accuracy_test.csv -&gt; ../../tests/results/tof_accuracy_test.csv"/>
-    <hyperlink ref="K18" r:id="rId42" tooltip="tof_accuracy_collect.py -&gt; ../../tests/scripts/tof_accuracy_collect.py"/>
-    <hyperlink ref="H19" r:id="rId43" tooltip="hardware/pcb/README.md -&gt; ../../hardware/pcb/README.md"/>
-    <hyperlink ref="H20" r:id="rId44" tooltip="power_brownout_test.csv -&gt; ../../tests/results/power_brownout_test.csv"/>
-    <hyperlink ref="I20" r:id="rId45" tooltip="power_brownout_test.py -&gt; ../../tests/scripts/power_brownout_test.py"/>
-    <hyperlink ref="H21" r:id="rId46" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="I21" r:id="rId47" tooltip="main -&gt; ../../firmware/main"/>
-    <hyperlink ref="J21" r:id="rId48" tooltip="cam -&gt; ../../firmware/camera/sketch_jan17a"/>
-    <hyperlink ref="H22" r:id="rId49" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="H23" r:id="rId50" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="I23" r:id="rId51" tooltip="web handlers -&gt; ../../firmware/main/03_WebHandlers.ino"/>
-    <hyperlink ref="J23" r:id="rId52" tooltip="tof_accuracy_test.csv -&gt; ../../tests/results/tof_accuracy_test.csv"/>
-    <hyperlink ref="H24" r:id="rId53" tooltip="camera firmware -&gt; ../../firmware/camera/sketch_jan17a/sketch_jan17a.ino"/>
-    <hyperlink ref="I24" r:id="rId54" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="H25" r:id="rId55" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="H28" r:id="rId56" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
-    <hyperlink ref="H29" r:id="rId57" tooltip="hardware/cad/ver3 -&gt; ../../hardware/cad/ver3"/>
-    <hyperlink ref="I29" r:id="rId58" tooltip="hardware/cad/real -&gt; ../../hardware/cad/real"/>
-    <hyperlink ref="H30" r:id="rId59" tooltip="hardware/cad/real/README.md -&gt; ../../hardware/cad/real/README.md"/>
-    <hyperlink ref="H31" r:id="rId60" tooltip="main -&gt; ../../firmware/main"/>
-    <hyperlink ref="I31" r:id="rId61" tooltip="cam -&gt; ../../firmware/camera/sketch_jan17a"/>
-    <hyperlink ref="H36" r:id="rId62" tooltip="ASSEMBLY_GUIDE.md -&gt; ../guides/ASSEMBLY_GUIDE.md"/>
-    <hyperlink ref="H37" r:id="rId63" tooltip="README.md -&gt; ../../README.md"/>
-    <hyperlink ref="I37" r:id="rId64" tooltip="docs README -&gt; ../README.md"/>
-    <hyperlink ref="J37" r:id="rId65" tooltip="requirements tracker Excel -&gt; VERSTAPOST_REQUIREMENTS_TRACKER.xlsx"/>
-    <hyperlink ref="H38" r:id="rId66" tooltip="requirements tracker Excel -&gt; VERSTAPOST_REQUIREMENTS_TRACKER.xlsx"/>
-    <hyperlink ref="I38" r:id="rId67" tooltip="docs index -&gt; ../README.md"/>
-    <hyperlink ref="H39" r:id="rId68" tooltip="FLASHING_GUIDE.md -&gt; ../guides/FLASHING_GUIDE.md"/>
-    <hyperlink ref="I39" r:id="rId69" tooltip="main -&gt; ../../firmware/main"/>
-    <hyperlink ref="J39" r:id="rId70" tooltip="camera firmware -&gt; ../../firmware/camera/sketch_jan17a/sketch_jan17a.ino"/>
-    <hyperlink ref="H40" r:id="rId71" tooltip="cad -&gt; ../../hardware/cad"/>
-    <hyperlink ref="I40" r:id="rId72" tooltip="hardware/cad/real -&gt; ../../hardware/cad/real"/>
-    <hyperlink ref="J40" r:id="rId73" tooltip="hardware/pcb/README.md -&gt; ../../hardware/pcb/README.md"/>
-    <hyperlink ref="K40" r:id="rId74" tooltip="PRINT_SETTINGS.md -&gt; ../guides/PRINT_SETTINGS.md"/>
-    <hyperlink ref="H41" r:id="rId75" tooltip="requirements tracker Excel -&gt; VERSTAPOST_REQUIREMENTS_TRACKER.xlsx"/>
-    <hyperlink ref="I41" r:id="rId76" tooltip="VERSTAPOSTID_PLAN.md -&gt; VERSTAPOSTID_PLAN.md"/>
-    <hyperlink ref="H42" r:id="rId77" tooltip="ASSEMBLY_GUIDE.md -&gt; ../guides/ASSEMBLY_GUIDE.md"/>
-    <hyperlink ref="H43" r:id="rId78" tooltip="FLASHING_GUIDE.md -&gt; ../guides/FLASHING_GUIDE.md"/>
-    <hyperlink ref="H44" r:id="rId79" tooltip="PRINT_SETTINGS.md -&gt; ../guides/PRINT_SETTINGS.md"/>
-    <hyperlink ref="H45" r:id="rId80" tooltip="test_results_analysis.ipynb -&gt; ../../tests/notebooks/test_results_analysis.ipynb"/>
-    <hyperlink ref="I45" r:id="rId81" tooltip="http_latency_analysis.ipynb -&gt; ../../tests/notebooks/http_latency_analysis.ipynb"/>
+    <hyperlink ref="H2" ns1:id="rId1" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
+    <hyperlink ref="I2" ns1:id="rId2" tooltip="Versta1.png -&gt; ../assets/briefs/Versta1.png"/>
+    <hyperlink ref="H3" ns1:id="rId3" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
+    <hyperlink ref="I3" ns1:id="rId4" tooltip="system_block.drawio.png -&gt; ../../hardware/diagrams/system_block.drawio.png"/>
+    <hyperlink ref="H4" ns1:id="rId5" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
+    <hyperlink ref="I4" ns1:id="rId6" tooltip="TECH_COMPARISON.md -&gt; ../specification/TECH_COMPARISON.md"/>
+    <hyperlink ref="H5" ns1:id="rId7" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
+    <hyperlink ref="H6" ns1:id="rId8" tooltip="V1_specification.md -&gt; ../specification/V1_specification.md"/>
+    <hyperlink ref="H7" ns1:id="rId9" tooltip="BOM.csv -&gt; ../specification/BOM.csv"/>
+    <hyperlink ref="I7" ns1:id="rId10" tooltip="Order1.png -&gt; ../assets/orders/Order1.png"/>
+    <hyperlink ref="J7" ns1:id="rId11" tooltip="Order2.png -&gt; ../assets/orders/Order2.png"/>
+    <hyperlink ref="H8" ns1:id="rId12" tooltip="power_scheme.md -&gt; ../specification/power_scheme.md"/>
+    <hyperlink ref="I8" ns1:id="rId13" tooltip="power_tree.drawio.png -&gt; ../../hardware/diagrams/power_tree.drawio.png"/>
+    <hyperlink ref="J8" ns1:id="rId14" tooltip="power_brownout_test.csv -&gt; ../../tests/results/power_brownout_test.csv"/>
+    <hyperlink ref="H9" ns1:id="rId15" tooltip="test_plan.md -&gt; ../testing/test_plan.md"/>
+    <hyperlink ref="H10" ns1:id="rId16" tooltip="hardware/cad/ver1 -&gt; ../../hardware/cad/ver1"/>
+    <hyperlink ref="I10" ns1:id="rId17" tooltip="hardware/pcb/README.md -&gt; ../../hardware/pcb/README.md"/>
+    <hyperlink ref="J10" ns1:id="rId18" tooltip="main -&gt; ../../firmware/main"/>
+    <hyperlink ref="K10" ns1:id="rId19" tooltip="cam -&gt; ../../firmware/camera/sketch_jan17a"/>
+    <hyperlink ref="H11" ns1:id="rId20" tooltip="TECH_COMPARISON.md -&gt; ../specification/TECH_COMPARISON.md"/>
+    <hyperlink ref="I11" ns1:id="rId21" tooltip="Vordlev_analyys_summary.md -&gt; ../analysis/Vordlev_analyys_summary.md"/>
+    <hyperlink ref="J11" ns1:id="rId22" tooltip="Vordlev_analyys.docx -&gt; ../analysis/Vordlev_analyys.docx"/>
+    <hyperlink ref="H12" ns1:id="rId23" tooltip="main firmware -&gt; ../../firmware/main/main.ino"/>
+    <hyperlink ref="I12" ns1:id="rId24" tooltip="web UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="J12" ns1:id="rId25" tooltip="motion logic -&gt; ../../firmware/main/02_Motion.ino"/>
+    <hyperlink ref="H13" ns1:id="rId26" tooltip="main firmware -&gt; ../../firmware/main/main.ino"/>
+    <hyperlink ref="I13" ns1:id="rId27" tooltip="web handlers -&gt; ../../firmware/main/03_WebHandlers.ino"/>
+    <hyperlink ref="H14" ns1:id="rId28" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="I14" ns1:id="rId29" tooltip="movement_speed_test.csv -&gt; ../../tests/results/movement_speed_test.csv"/>
+    <hyperlink ref="H15" ns1:id="rId30" tooltip="movement_speed_test.csv -&gt; ../../tests/results/movement_speed_test.csv"/>
+    <hyperlink ref="I15" ns1:id="rId31" tooltip="movement_drift_test.csv -&gt; ../../tests/results/movement_drift_test.csv"/>
+    <hyperlink ref="J15" ns1:id="rId32" tooltip="movement_turn_test.csv -&gt; ../../tests/results/movement_turn_test.csv"/>
+    <hyperlink ref="K15" ns1:id="rId33" tooltip="tof_stop_test.csv -&gt; ../../tests/results/tof_stop_test.csv"/>
+    <hyperlink ref="H16" ns1:id="rId34" tooltip="http_latency_analysis.ipynb -&gt; ../../tests/notebooks/http_latency_analysis.ipynb"/>
+    <hyperlink ref="I16" ns1:id="rId35" tooltip="latency_test_result.md -&gt; ../testing/latency_test_result.md"/>
+    <hyperlink ref="J16" ns1:id="rId36" tooltip="test_results_analysis.ipynb -&gt; ../../tests/notebooks/test_results_analysis.ipynb"/>
+    <hyperlink ref="H17" ns1:id="rId37" tooltip="camera firmware -&gt; ../../firmware/camera/sketch_jan17a/sketch_jan17a.ino"/>
+    <hyperlink ref="I17" ns1:id="rId38" tooltip="demo video -&gt; ../../media/video/MicrosoftTeams-video.mp4"/>
+    <hyperlink ref="H18" ns1:id="rId39" tooltip="main firmware -&gt; ../../firmware/main/main.ino"/>
+    <hyperlink ref="I18" ns1:id="rId40" tooltip="tof_stop_test.csv -&gt; ../../tests/results/tof_stop_test.csv"/>
+    <hyperlink ref="J18" ns1:id="rId41" tooltip="tof_accuracy_test.csv -&gt; ../../tests/results/tof_accuracy_test.csv"/>
+    <hyperlink ref="K18" ns1:id="rId42" tooltip="tof_accuracy_collect.py -&gt; ../../tests/scripts/tof_accuracy_collect.py"/>
+    <hyperlink ref="H19" ns1:id="rId43" tooltip="hardware/pcb/README.md -&gt; ../../hardware/pcb/README.md"/>
+    <hyperlink ref="H20" ns1:id="rId44" tooltip="power_brownout_test.csv -&gt; ../../tests/results/power_brownout_test.csv"/>
+    <hyperlink ref="I20" ns1:id="rId45" tooltip="power_brownout_test.py -&gt; ../../tests/scripts/power_brownout_test.py"/>
+    <hyperlink ref="H21" ns1:id="rId46" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="I21" ns1:id="rId47" tooltip="main -&gt; ../../firmware/main"/>
+    <hyperlink ref="J21" ns1:id="rId48" tooltip="cam -&gt; ../../firmware/camera/sketch_jan17a"/>
+    <hyperlink ref="H22" ns1:id="rId49" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="H23" ns1:id="rId50" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="I23" ns1:id="rId51" tooltip="web handlers -&gt; ../../firmware/main/03_WebHandlers.ino"/>
+    <hyperlink ref="J23" ns1:id="rId52" tooltip="tof_accuracy_test.csv -&gt; ../../tests/results/tof_accuracy_test.csv"/>
+    <hyperlink ref="H24" ns1:id="rId53" tooltip="camera firmware -&gt; ../../firmware/camera/sketch_jan17a/sketch_jan17a.ino"/>
+    <hyperlink ref="I24" ns1:id="rId54" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="H25" ns1:id="rId55" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="H28" ns1:id="rId56" tooltip="main UI -&gt; ../../firmware/main/01_WebUi.ino"/>
+    <hyperlink ref="H29" ns1:id="rId57" tooltip="hardware/cad/ver3 -&gt; ../../hardware/cad/ver3"/>
+    <hyperlink ref="I29" ns1:id="rId58" tooltip="hardware/cad/real -&gt; ../../hardware/cad/real"/>
+    <hyperlink ref="H30" ns1:id="rId59" tooltip="hardware/cad/real/README.md -&gt; ../../hardware/cad/real/README.md"/>
+    <hyperlink ref="H31" ns1:id="rId60" tooltip="main -&gt; ../../firmware/main"/>
+    <hyperlink ref="I31" ns1:id="rId61" tooltip="cam -&gt; ../../firmware/camera/sketch_jan17a"/>
+    <hyperlink ref="H36" ns1:id="rId62" tooltip="ASSEMBLY_GUIDE.md -&gt; ../guides/ASSEMBLY_GUIDE.md"/>
+    <hyperlink ref="H37" ns1:id="rId63" tooltip="README.md -&gt; ../../README.md"/>
+    <hyperlink ref="I37" ns1:id="rId64" tooltip="docs README -&gt; ../README.md"/>
+    <hyperlink ref="J37" ns1:id="rId65" tooltip="requirements tracker Excel -&gt; VERSTAPOST_REQUIREMENTS_TRACKER.xlsx"/>
+    <hyperlink ref="H38" ns1:id="rId66" tooltip="requirements tracker Excel -&gt; VERSTAPOST_REQUIREMENTS_TRACKER.xlsx"/>
+    <hyperlink ref="I38" ns1:id="rId67" tooltip="docs index -&gt; ../README.md"/>
+    <hyperlink ref="H39" ns1:id="rId68" tooltip="FLASHING_GUIDE.md -&gt; ../guides/FLASHING_GUIDE.md"/>
+    <hyperlink ref="I39" ns1:id="rId69" tooltip="main -&gt; ../../firmware/main"/>
+    <hyperlink ref="J39" ns1:id="rId70" tooltip="camera firmware -&gt; ../../firmware/camera/sketch_jan17a/sketch_jan17a.ino"/>
+    <hyperlink ref="H40" ns1:id="rId71" tooltip="cad -&gt; ../../hardware/cad"/>
+    <hyperlink ref="I40" ns1:id="rId72" tooltip="hardware/cad/real -&gt; ../../hardware/cad/real"/>
+    <hyperlink ref="J40" ns1:id="rId73" tooltip="hardware/pcb/README.md -&gt; ../../hardware/pcb/README.md"/>
+    <hyperlink ref="K40" ns1:id="rId74" tooltip="PRINT_SETTINGS.md -&gt; ../guides/PRINT_SETTINGS.md"/>
+    <hyperlink ref="H41" ns1:id="rId75" tooltip="requirements tracker Excel -&gt; VERSTAPOST_REQUIREMENTS_TRACKER.xlsx"/>
+    <hyperlink ref="I41" ns1:id="rId76" tooltip="VERSTAPOSTID_PLAN.md -&gt; VERSTAPOSTID_PLAN.md"/>
+    <hyperlink ref="H42" ns1:id="rId77" tooltip="ASSEMBLY_GUIDE.md -&gt; ../guides/ASSEMBLY_GUIDE.md"/>
+    <hyperlink ref="H43" ns1:id="rId78" tooltip="FLASHING_GUIDE.md -&gt; ../guides/FLASHING_GUIDE.md"/>
+    <hyperlink ref="H44" ns1:id="rId79" tooltip="PRINT_SETTINGS.md -&gt; ../guides/PRINT_SETTINGS.md"/>
+    <hyperlink ref="H45" ns1:id="rId80" tooltip="test_results_analysis.ipynb -&gt; ../../tests/notebooks/test_results_analysis.ipynb"/>
+    <hyperlink ref="I45" ns1:id="rId81" tooltip="http_latency_analysis.ipynb -&gt; ../../tests/notebooks/http_latency_analysis.ipynb"/>
+    <hyperlink ref="L18" ns1:id="rId82" tooltip="ToF calibration note -&gt; ../testing/tof_calibration_note.md"/>
+    <hyperlink ref="I19" ns1:id="rId83" tooltip="PCB evidence check -&gt; ../../hardware/pcb/PCB_EVIDENCE_CHECK.md"/>
+    <hyperlink ref="J20" ns1:id="rId84" tooltip="Power brownout analysis -&gt; ../testing/power_brownout_analysis.md"/>
   </hyperlinks>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G9"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -3232,14 +3235,20 @@
       <c r="B3">
         <v>9</v>
       </c>
-      <c r="C3">
-        <v>6</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3261,18 +3270,24 @@
       <c r="B4">
         <v>8</v>
       </c>
-      <c r="C4">
-        <v>4</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Ready with gaps</t>
+          <t>Ready with gap</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">

</xml_diff>